<commit_message>
chore(excel): update graph generation script
</commit_message>
<xml_diff>
--- a/notebooks/exported_graphs.xlsx
+++ b/notebooks/exported_graphs.xlsx
@@ -11,6 +11,7 @@
     <sheet name="SOH Degradation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Physics vs Measured Cell1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Pred vs Measured Test" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="OOD Pred vs Measured" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -227,6 +228,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>70</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="6791325"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -300,6 +326,36 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="7620000" cy="7591425"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7620000" cy="7543800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -609,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +700,13 @@
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Pred vs Measured Test</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>OOD Pred vs Measured</t>
         </is>
       </c>
     </row>
@@ -8799,4 +8862,583 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OOD Pred vs Measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Source data</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>measured_soh</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>physics_pred</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>hybrid_pinn_pred</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0.618</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.747</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.757</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>0.745</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.749</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.774</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="B38" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.786</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="B41" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.794</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="B42" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.796</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="B43" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.794</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="B44" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.792</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="B46" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.788</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="B47" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="B48" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.766</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="B49" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.772</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="B50" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.776</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="B51" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="B52" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.784</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="B53" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.786</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="B54" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.788</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="B55" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.786</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="B56" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.782</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="B57" t="n">
+        <v>0.752</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="B58" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.756</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>0.804</v>
+      </c>
+      <c r="B59" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.762</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="B60" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="B61" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.774</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="B62" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.778</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="B63" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.782</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="B64" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0.786</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="B65" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0.788</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B66" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0.752</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0.758</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0.764</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0.776</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0.784</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="B73" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0.788</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="B74" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0.766</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="B75" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0.778</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="B76" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0.784</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="B77" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0.782</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="B78" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0.776</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="B79" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="B80" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0.764</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>